<commit_message>
feat : Addressable 적용 단계
</commit_message>
<xml_diff>
--- a/Assets/Editor/ExcelData/MatchDropData.xlsx
+++ b/Assets/Editor/ExcelData/MatchDropData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\SHINZI_Games_InternshipTest\Assets\Editor\ExcelData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C48E999-A7B9-4976-8A0D-D590F904D8CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7E3A726-6B49-480D-9943-B1B2840054E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="43080" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{26BA0CAA-DEB9-4337-88BD-7920261670E1}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{26BA0CAA-DEB9-4337-88BD-7920261670E1}"/>
   </bookViews>
   <sheets>
     <sheet name="MatchDropData" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="11">
   <si>
     <t>weaponId</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -73,19 +73,15 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>Arrow</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Melee</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>Hammer</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>Shield</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Bow</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -498,7 +494,7 @@
         <v>6</v>
       </c>
       <c r="B2" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C2">
         <v>2</v>
@@ -520,7 +516,7 @@
         <v>6</v>
       </c>
       <c r="B4" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C4">
         <v>3</v>
@@ -531,7 +527,7 @@
         <v>6</v>
       </c>
       <c r="B5" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C5">
         <v>4</v>
@@ -564,7 +560,7 @@
         <v>5</v>
       </c>
       <c r="B8" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C8">
         <v>4</v>
@@ -575,7 +571,7 @@
         <v>5</v>
       </c>
       <c r="B9" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C9">
         <v>2</v>
@@ -597,7 +593,7 @@
         <v>4</v>
       </c>
       <c r="B11" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C11">
         <v>3</v>
@@ -608,7 +604,7 @@
         <v>4</v>
       </c>
       <c r="B12" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C12">
         <v>3</v>

</xml_diff>